<commit_message>
Veri Görselleştirme İşlemleri Yapıldı
</commit_message>
<xml_diff>
--- a/cleaned_data.xlsx
+++ b/cleaned_data.xlsx
@@ -2868,7 +2868,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr"/>
+      <c r="S30" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3271,7 +3273,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S35" t="inlineStr"/>
+      <c r="S35" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4320,7 +4324,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr"/>
+      <c r="S48" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5209,7 +5215,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S59" t="inlineStr"/>
+      <c r="S59" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6467,7 +6475,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -6744,7 +6752,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S78" t="inlineStr"/>
+      <c r="S78" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6985,7 +6995,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S81" t="inlineStr"/>
+      <c r="S81" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7064,7 +7076,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S82" t="inlineStr"/>
+      <c r="S82" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7305,7 +7319,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S85" t="inlineStr"/>
+      <c r="S85" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -8032,7 +8048,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S94" t="inlineStr"/>
+      <c r="S94" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8644,7 +8662,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -8759,7 +8777,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S103" t="inlineStr"/>
+      <c r="S103" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8804,7 +8824,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -8838,7 +8858,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S104" t="inlineStr"/>
+      <c r="S104" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9610,7 +9632,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -9644,7 +9666,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S114" t="inlineStr"/>
+      <c r="S114" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -10047,7 +10071,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S119" t="inlineStr"/>
+      <c r="S119" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -10207,7 +10233,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S121" t="inlineStr"/>
+      <c r="S121" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -12473,7 +12501,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S149" t="inlineStr"/>
+      <c r="S149" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -12552,7 +12582,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S150" t="inlineStr"/>
+      <c r="S150" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -12631,7 +12663,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S151" t="inlineStr"/>
+      <c r="S151" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -12872,7 +12906,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S154" t="inlineStr"/>
+      <c r="S154" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -12951,7 +12987,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S155" t="inlineStr"/>
+      <c r="S155" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -13354,7 +13392,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S160" t="inlineStr"/>
+      <c r="S160" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -14000,7 +14040,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S168" t="inlineStr"/>
+      <c r="S168" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -14160,7 +14202,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S170" t="inlineStr"/>
+      <c r="S170" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -14320,7 +14364,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S172" t="inlineStr"/>
+      <c r="S172" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -14561,7 +14607,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S175" t="inlineStr"/>
+      <c r="S175" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -14883,7 +14931,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S179" t="inlineStr"/>
+      <c r="S179" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -15043,7 +15093,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S181" t="inlineStr"/>
+      <c r="S181" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -15446,7 +15498,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S186" t="inlineStr"/>
+      <c r="S186" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -17064,7 +17118,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S206" t="inlineStr"/>
+      <c r="S206" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -17224,7 +17280,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S208" t="inlineStr"/>
+      <c r="S208" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -17303,7 +17361,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S209" t="inlineStr"/>
+      <c r="S209" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -17382,7 +17442,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S210" t="inlineStr"/>
+      <c r="S210" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -17542,7 +17604,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S212" t="inlineStr"/>
+      <c r="S212" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -17783,7 +17847,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S215" t="inlineStr"/>
+      <c r="S215" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -18024,7 +18090,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S218" t="inlineStr"/>
+      <c r="S218" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -18670,7 +18738,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S226" t="inlineStr"/>
+      <c r="S226" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -18911,7 +18981,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S229" t="inlineStr"/>
+      <c r="S229" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -18990,7 +19062,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S230" t="inlineStr"/>
+      <c r="S230" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -19357,7 +19431,7 @@
       </c>
       <c r="K235" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L235" t="inlineStr">
@@ -19472,7 +19546,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S236" t="inlineStr"/>
+      <c r="S236" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -19517,7 +19593,7 @@
       </c>
       <c r="K237" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L237" t="inlineStr">
@@ -19956,7 +20032,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S242" t="inlineStr"/>
+      <c r="S242" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -20440,7 +20518,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S248" t="inlineStr"/>
+      <c r="S248" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -22781,7 +22861,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S277" t="inlineStr"/>
+      <c r="S277" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -23022,7 +23104,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S280" t="inlineStr"/>
+      <c r="S280" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -23263,7 +23347,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S283" t="inlineStr"/>
+      <c r="S283" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -24314,7 +24400,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S296" t="inlineStr"/>
+      <c r="S296" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -24393,7 +24481,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S297" t="inlineStr"/>
+      <c r="S297" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -24634,7 +24724,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S300" t="inlineStr"/>
+      <c r="S300" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -24794,7 +24886,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S302" t="inlineStr"/>
+      <c r="S302" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -25035,7 +25129,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S305" t="inlineStr"/>
+      <c r="S305" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -25276,7 +25372,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S308" t="inlineStr"/>
+      <c r="S308" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -25841,7 +25939,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S315" t="inlineStr"/>
+      <c r="S315" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -26325,7 +26425,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S321" t="inlineStr"/>
+      <c r="S321" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -26485,7 +26587,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S323" t="inlineStr"/>
+      <c r="S323" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -27739,7 +27843,7 @@
       </c>
       <c r="K339" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L339" t="inlineStr">
@@ -27935,7 +28039,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S341" t="inlineStr"/>
+      <c r="S341" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -28419,7 +28525,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S347" t="inlineStr"/>
+      <c r="S347" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -28498,7 +28606,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S348" t="inlineStr"/>
+      <c r="S348" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -28577,7 +28687,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S349" t="inlineStr"/>
+      <c r="S349" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -28737,7 +28849,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S351" t="inlineStr"/>
+      <c r="S351" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -29219,7 +29333,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S357" t="inlineStr"/>
+      <c r="S357" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -29541,7 +29657,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S361" t="inlineStr"/>
+      <c r="S361" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -29584,7 +29702,7 @@
       </c>
       <c r="K362" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L362" t="inlineStr">
@@ -29942,7 +30060,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S366" t="inlineStr"/>
+      <c r="S366" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -30021,7 +30141,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S367" t="inlineStr"/>
+      <c r="S367" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -30262,7 +30384,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S370" t="inlineStr"/>
+      <c r="S370" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -30422,7 +30546,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S372" t="inlineStr"/>
+      <c r="S372" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -30663,7 +30789,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S375" t="inlineStr"/>
+      <c r="S375" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -31309,7 +31437,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S383" t="inlineStr"/>
+      <c r="S383" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -31435,7 +31565,7 @@
       </c>
       <c r="K385" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L385" t="inlineStr">
@@ -31712,7 +31842,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S388" t="inlineStr"/>
+      <c r="S388" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -31791,7 +31923,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S389" t="inlineStr"/>
+      <c r="S389" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -31951,7 +32085,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S391" t="inlineStr"/>
+      <c r="S391" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -32435,7 +32571,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S397" t="inlineStr"/>
+      <c r="S397" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -32514,7 +32652,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S398" t="inlineStr"/>
+      <c r="S398" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -32593,7 +32733,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S399" t="inlineStr"/>
+      <c r="S399" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -33039,7 +33181,7 @@
       </c>
       <c r="K405" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L405" t="inlineStr">
@@ -33316,7 +33458,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S408" t="inlineStr"/>
+      <c r="S408" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -33962,7 +34106,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S416" t="inlineStr"/>
+      <c r="S416" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -34122,7 +34268,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S418" t="inlineStr"/>
+      <c r="S418" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -34489,7 +34637,7 @@
       </c>
       <c r="K423" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L423" t="inlineStr">
@@ -34928,7 +35076,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S428" t="inlineStr"/>
+      <c r="S428" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -35167,7 +35317,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S431" t="inlineStr"/>
+      <c r="S431" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -35327,7 +35479,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S433" t="inlineStr"/>
+      <c r="S433" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -35406,7 +35560,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S434" t="inlineStr"/>
+      <c r="S434" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -35647,7 +35803,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S437" t="inlineStr"/>
+      <c r="S437" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -35888,7 +36046,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S440" t="inlineStr"/>
+      <c r="S440" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -36174,7 +36334,7 @@
       </c>
       <c r="K444" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L444" t="inlineStr">
@@ -36775,7 +36935,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S451" t="inlineStr"/>
+      <c r="S451" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -37016,7 +37178,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S454" t="inlineStr"/>
+      <c r="S454" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -37095,7 +37259,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S455" t="inlineStr"/>
+      <c r="S455" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -37496,7 +37662,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S460" t="inlineStr"/>
+      <c r="S460" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -37656,7 +37824,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S462" t="inlineStr"/>
+      <c r="S462" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -37816,7 +37986,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S464" t="inlineStr"/>
+      <c r="S464" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -38183,7 +38355,7 @@
       </c>
       <c r="K469" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L469" t="inlineStr">
@@ -38298,7 +38470,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S470" t="inlineStr"/>
+      <c r="S470" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -38377,7 +38551,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S471" t="inlineStr"/>
+      <c r="S471" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -38537,7 +38713,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S473" t="inlineStr"/>
+      <c r="S473" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -38697,7 +38875,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S475" t="inlineStr"/>
+      <c r="S475" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -38938,7 +39118,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S478" t="inlineStr"/>
+      <c r="S478" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -39501,7 +39683,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S485" t="inlineStr"/>
+      <c r="S485" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -39902,7 +40086,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S490" t="inlineStr"/>
+      <c r="S490" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -40222,7 +40408,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S494" t="inlineStr"/>
+      <c r="S494" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -40463,7 +40651,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S497" t="inlineStr"/>
+      <c r="S497" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -40542,7 +40732,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S498" t="inlineStr"/>
+      <c r="S498" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -40585,7 +40777,7 @@
       </c>
       <c r="K499" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L499" t="inlineStr">
@@ -40781,7 +40973,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S501" t="inlineStr"/>
+      <c r="S501" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -41265,7 +41459,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S507" t="inlineStr"/>
+      <c r="S507" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
@@ -41425,7 +41621,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S509" t="inlineStr"/>
+      <c r="S509" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -41828,7 +42026,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S514" t="inlineStr"/>
+      <c r="S514" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -41907,7 +42107,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S515" t="inlineStr"/>
+      <c r="S515" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
@@ -42355,7 +42557,7 @@
       </c>
       <c r="K521" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L521" t="inlineStr">
@@ -42758,7 +42960,7 @@
       </c>
       <c r="K526" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L526" t="inlineStr">
@@ -43519,7 +43721,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S535" t="inlineStr"/>
+      <c r="S535" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
@@ -44244,7 +44448,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S544" t="inlineStr"/>
+      <c r="S544" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -44566,7 +44772,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S548" t="inlineStr"/>
+      <c r="S548" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
@@ -44888,7 +45096,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S552" t="inlineStr"/>
+      <c r="S552" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="553">
       <c r="A553" t="inlineStr">
@@ -45129,7 +45339,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S555" t="inlineStr"/>
+      <c r="S555" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
@@ -45289,7 +45501,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S557" t="inlineStr"/>
+      <c r="S557" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
@@ -45530,7 +45744,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S560" t="inlineStr"/>
+      <c r="S560" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
@@ -45654,7 +45870,7 @@
       </c>
       <c r="K562" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L562" t="inlineStr">
@@ -46336,7 +46552,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S570" t="inlineStr"/>
+      <c r="S570" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
@@ -46577,7 +46795,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S573" t="inlineStr"/>
+      <c r="S573" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
@@ -46980,7 +47200,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S578" t="inlineStr"/>
+      <c r="S578" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
@@ -47221,7 +47443,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S581" t="inlineStr"/>
+      <c r="S581" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="582">
       <c r="A582" t="inlineStr">
@@ -47381,7 +47605,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S583" t="inlineStr"/>
+      <c r="S583" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
@@ -47460,7 +47686,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S584" t="inlineStr"/>
+      <c r="S584" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
@@ -48106,7 +48334,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S592" t="inlineStr"/>
+      <c r="S592" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
@@ -48185,7 +48415,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S593" t="inlineStr"/>
+      <c r="S593" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
@@ -48588,7 +48820,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S598" t="inlineStr"/>
+      <c r="S598" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
@@ -48829,7 +49063,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S601" t="inlineStr"/>
+      <c r="S601" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
@@ -48908,7 +49144,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S602" t="inlineStr"/>
+      <c r="S602" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
@@ -49066,7 +49304,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S604" t="inlineStr"/>
+      <c r="S604" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
@@ -49145,7 +49385,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S605" t="inlineStr"/>
+      <c r="S605" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
@@ -49305,7 +49547,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S607" t="inlineStr"/>
+      <c r="S607" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
@@ -49627,7 +49871,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S611" t="inlineStr"/>
+      <c r="S611" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
@@ -50030,7 +50276,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S616" t="inlineStr"/>
+      <c r="S616" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
@@ -50271,7 +50519,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S619" t="inlineStr"/>
+      <c r="S619" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
@@ -50350,7 +50600,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S620" t="inlineStr"/>
+      <c r="S620" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
@@ -50510,7 +50762,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S622" t="inlineStr"/>
+      <c r="S622" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
@@ -50751,7 +51005,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S625" t="inlineStr"/>
+      <c r="S625" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="626">
       <c r="A626" t="inlineStr">
@@ -50830,7 +51086,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S626" t="inlineStr"/>
+      <c r="S626" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="627">
       <c r="A627" t="inlineStr">
@@ -51152,7 +51410,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S630" t="inlineStr"/>
+      <c r="S630" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="631">
       <c r="A631" t="inlineStr">
@@ -51393,7 +51653,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S633" t="inlineStr"/>
+      <c r="S633" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="634">
       <c r="A634" t="inlineStr">
@@ -51472,7 +51734,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S634" t="inlineStr"/>
+      <c r="S634" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
@@ -51632,7 +51896,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S636" t="inlineStr"/>
+      <c r="S636" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
@@ -51954,7 +52220,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S640" t="inlineStr"/>
+      <c r="S640" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
@@ -52114,7 +52382,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S642" t="inlineStr"/>
+      <c r="S642" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
@@ -52193,7 +52463,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S643" t="inlineStr"/>
+      <c r="S643" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
@@ -52238,7 +52510,7 @@
       </c>
       <c r="K644" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L644" t="inlineStr">
@@ -52515,7 +52787,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S647" t="inlineStr"/>
+      <c r="S647" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr">
@@ -52594,7 +52868,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S648" t="inlineStr"/>
+      <c r="S648" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
@@ -52754,7 +53030,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S650" t="inlineStr"/>
+      <c r="S650" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
@@ -52833,7 +53111,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S651" t="inlineStr"/>
+      <c r="S651" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
@@ -53074,7 +53354,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S654" t="inlineStr"/>
+      <c r="S654" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
@@ -53117,7 +53399,7 @@
       </c>
       <c r="K655" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L655" t="inlineStr">
@@ -53313,7 +53595,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S657" t="inlineStr"/>
+      <c r="S657" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr">
@@ -53392,7 +53676,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S658" t="inlineStr"/>
+      <c r="S658" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr">
@@ -53471,7 +53757,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S659" t="inlineStr"/>
+      <c r="S659" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="660">
       <c r="A660" t="inlineStr">
@@ -53550,7 +53838,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S660" t="inlineStr"/>
+      <c r="S660" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
@@ -53629,7 +53919,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S661" t="inlineStr"/>
+      <c r="S661" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr">
@@ -53789,7 +54081,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S663" t="inlineStr"/>
+      <c r="S663" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="664">
       <c r="A664" t="inlineStr">
@@ -54111,7 +54405,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S667" t="inlineStr"/>
+      <c r="S667" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="668">
       <c r="A668" t="inlineStr">
@@ -54190,7 +54486,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S668" t="inlineStr"/>
+      <c r="S668" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="669">
       <c r="A669" t="inlineStr">
@@ -54269,7 +54567,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S669" t="inlineStr"/>
+      <c r="S669" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="670">
       <c r="A670" t="inlineStr">
@@ -54753,7 +55053,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S675" t="inlineStr"/>
+      <c r="S675" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="676">
       <c r="A676" t="inlineStr">
@@ -54992,7 +55294,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S678" t="inlineStr"/>
+      <c r="S678" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="679">
       <c r="A679" t="inlineStr">
@@ -55071,7 +55375,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S679" t="inlineStr"/>
+      <c r="S679" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="680">
       <c r="A680" t="inlineStr">
@@ -55231,7 +55537,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S681" t="inlineStr"/>
+      <c r="S681" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="682">
       <c r="A682" t="inlineStr">
@@ -55310,7 +55618,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S682" t="inlineStr"/>
+      <c r="S682" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="683">
       <c r="A683" t="inlineStr">
@@ -55389,7 +55699,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S683" t="inlineStr"/>
+      <c r="S683" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="684">
       <c r="A684" t="inlineStr">
@@ -55954,7 +56266,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S690" t="inlineStr"/>
+      <c r="S690" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="691">
       <c r="A691" t="inlineStr">
@@ -56033,7 +56347,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S691" t="inlineStr"/>
+      <c r="S691" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="692">
       <c r="A692" t="inlineStr">
@@ -56112,7 +56428,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S692" t="inlineStr"/>
+      <c r="S692" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="693">
       <c r="A693" t="inlineStr">
@@ -56155,7 +56473,7 @@
       </c>
       <c r="K693" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L693" t="inlineStr">
@@ -56268,7 +56586,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S694" t="inlineStr"/>
+      <c r="S694" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="695">
       <c r="A695" t="inlineStr">
@@ -56426,7 +56746,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S696" t="inlineStr"/>
+      <c r="S696" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="697">
       <c r="A697" t="inlineStr">
@@ -56471,7 +56793,7 @@
       </c>
       <c r="K697" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L697" t="inlineStr">
@@ -56586,7 +56908,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S698" t="inlineStr"/>
+      <c r="S698" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="699">
       <c r="A699" t="inlineStr">
@@ -56665,7 +56989,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S699" t="inlineStr"/>
+      <c r="S699" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="700">
       <c r="A700" t="inlineStr">
@@ -56825,7 +57151,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S701" t="inlineStr"/>
+      <c r="S701" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="702">
       <c r="A702" t="inlineStr">
@@ -56985,7 +57313,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S703" t="inlineStr"/>
+      <c r="S703" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="704">
       <c r="A704" t="inlineStr">
@@ -57064,7 +57394,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S704" t="inlineStr"/>
+      <c r="S704" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="705">
       <c r="A705" t="inlineStr">
@@ -57465,7 +57797,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S709" t="inlineStr"/>
+      <c r="S709" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="710">
       <c r="A710" t="inlineStr">
@@ -57544,7 +57878,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S710" t="inlineStr"/>
+      <c r="S710" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="711">
       <c r="A711" t="inlineStr">
@@ -57623,7 +57959,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S711" t="inlineStr"/>
+      <c r="S711" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="712">
       <c r="A712" t="inlineStr">
@@ -57783,7 +58121,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S713" t="inlineStr"/>
+      <c r="S713" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="714">
       <c r="A714" t="inlineStr">
@@ -58105,7 +58445,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S717" t="inlineStr"/>
+      <c r="S717" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="718">
       <c r="A718" t="inlineStr">
@@ -58265,7 +58607,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S719" t="inlineStr"/>
+      <c r="S719" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="720">
       <c r="A720" t="inlineStr">
@@ -58344,7 +58688,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S720" t="inlineStr"/>
+      <c r="S720" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="721">
       <c r="A721" t="inlineStr">
@@ -58585,7 +58931,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S723" t="inlineStr"/>
+      <c r="S723" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="724">
       <c r="A724" t="inlineStr">
@@ -58664,7 +59012,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S724" t="inlineStr"/>
+      <c r="S724" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="725">
       <c r="A725" t="inlineStr">
@@ -59229,7 +59579,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S731" t="inlineStr"/>
+      <c r="S731" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="732">
       <c r="A732" t="inlineStr">
@@ -59308,7 +59660,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S732" t="inlineStr"/>
+      <c r="S732" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="733">
       <c r="A733" t="inlineStr">
@@ -59468,7 +59822,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S734" t="inlineStr"/>
+      <c r="S734" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr">
@@ -59547,7 +59903,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S735" t="inlineStr"/>
+      <c r="S735" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="736">
       <c r="A736" t="inlineStr">
@@ -59626,7 +59984,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S736" t="inlineStr"/>
+      <c r="S736" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="737">
       <c r="A737" t="inlineStr">
@@ -59705,7 +60065,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S737" t="inlineStr"/>
+      <c r="S737" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="738">
       <c r="A738" t="inlineStr">
@@ -59863,7 +60225,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S739" t="inlineStr"/>
+      <c r="S739" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="740">
       <c r="A740" t="inlineStr">
@@ -59942,7 +60306,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S740" t="inlineStr"/>
+      <c r="S740" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="741">
       <c r="A741" t="inlineStr">
@@ -60021,7 +60387,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S741" t="inlineStr"/>
+      <c r="S741" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="742">
       <c r="A742" t="inlineStr">
@@ -60100,7 +60468,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S742" t="inlineStr"/>
+      <c r="S742" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="743">
       <c r="A743" t="inlineStr">
@@ -60179,7 +60549,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S743" t="inlineStr"/>
+      <c r="S743" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="744">
       <c r="A744" t="inlineStr">
@@ -60420,7 +60792,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S746" t="inlineStr"/>
+      <c r="S746" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="747">
       <c r="A747" t="inlineStr">
@@ -60580,7 +60954,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S748" t="inlineStr"/>
+      <c r="S748" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="749">
       <c r="A749" t="inlineStr">
@@ -60740,7 +61116,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S750" t="inlineStr"/>
+      <c r="S750" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="751">
       <c r="A751" t="inlineStr">
@@ -60864,7 +61242,7 @@
       </c>
       <c r="K752" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L752" t="inlineStr">
@@ -61060,7 +61438,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S754" t="inlineStr"/>
+      <c r="S754" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="755">
       <c r="A755" t="inlineStr">
@@ -61220,7 +61600,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S756" t="inlineStr"/>
+      <c r="S756" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="757">
       <c r="A757" t="inlineStr">
@@ -61380,7 +61762,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S758" t="inlineStr"/>
+      <c r="S758" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="759">
       <c r="A759" t="inlineStr">
@@ -61783,7 +62167,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S763" t="inlineStr"/>
+      <c r="S763" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="764">
       <c r="A764" t="inlineStr">
@@ -61862,7 +62248,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S764" t="inlineStr"/>
+      <c r="S764" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="765">
       <c r="A765" t="inlineStr">
@@ -61941,7 +62329,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S765" t="inlineStr"/>
+      <c r="S765" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="766">
       <c r="A766" t="inlineStr">
@@ -62020,7 +62410,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S766" t="inlineStr"/>
+      <c r="S766" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="767">
       <c r="A767" t="inlineStr">
@@ -62099,7 +62491,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S767" t="inlineStr"/>
+      <c r="S767" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="768">
       <c r="A768" t="inlineStr">
@@ -62178,7 +62572,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S768" t="inlineStr"/>
+      <c r="S768" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="769">
       <c r="A769" t="inlineStr">
@@ -62257,7 +62653,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S769" t="inlineStr"/>
+      <c r="S769" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="770">
       <c r="A770" t="inlineStr">
@@ -62336,7 +62734,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S770" t="inlineStr"/>
+      <c r="S770" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="771">
       <c r="A771" t="inlineStr">
@@ -62820,7 +63220,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S776" t="inlineStr"/>
+      <c r="S776" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="777">
       <c r="A777" t="inlineStr">
@@ -62899,7 +63301,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S777" t="inlineStr"/>
+      <c r="S777" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="778">
       <c r="A778" t="inlineStr">
@@ -62978,7 +63382,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S778" t="inlineStr"/>
+      <c r="S778" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="779">
       <c r="A779" t="inlineStr">
@@ -63057,7 +63463,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S779" t="inlineStr"/>
+      <c r="S779" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="780">
       <c r="A780" t="inlineStr">
@@ -63136,7 +63544,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S780" t="inlineStr"/>
+      <c r="S780" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="781">
       <c r="A781" t="inlineStr">
@@ -63296,7 +63706,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S782" t="inlineStr"/>
+      <c r="S782" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="783">
       <c r="A783" t="inlineStr">
@@ -63454,7 +63866,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S784" t="inlineStr"/>
+      <c r="S784" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="785">
       <c r="A785" t="inlineStr">
@@ -63533,7 +63947,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S785" t="inlineStr"/>
+      <c r="S785" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="786">
       <c r="A786" t="inlineStr">
@@ -63612,7 +64028,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S786" t="inlineStr"/>
+      <c r="S786" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="787">
       <c r="A787" t="inlineStr">
@@ -63772,7 +64190,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S788" t="inlineStr"/>
+      <c r="S788" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="789">
       <c r="A789" t="inlineStr">
@@ -63851,7 +64271,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S789" t="inlineStr"/>
+      <c r="S789" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="790">
       <c r="A790" t="inlineStr">
@@ -64092,7 +64514,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S792" t="inlineStr"/>
+      <c r="S792" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="793">
       <c r="A793" t="inlineStr">
@@ -64252,7 +64676,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S794" t="inlineStr"/>
+      <c r="S794" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -64491,7 +64917,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S797" t="inlineStr"/>
+      <c r="S797" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="798">
       <c r="A798" t="inlineStr">
@@ -65218,7 +65646,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S806" t="inlineStr"/>
+      <c r="S806" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="807">
       <c r="A807" t="inlineStr">
@@ -65297,7 +65727,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S807" t="inlineStr"/>
+      <c r="S807" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="808">
       <c r="A808" t="inlineStr">
@@ -65538,7 +65970,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S810" t="inlineStr"/>
+      <c r="S810" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="811">
       <c r="A811" t="inlineStr">
@@ -65698,7 +66132,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S812" t="inlineStr"/>
+      <c r="S812" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="813">
       <c r="A813" t="inlineStr">
@@ -65858,7 +66294,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S814" t="inlineStr"/>
+      <c r="S814" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="815">
       <c r="A815" t="inlineStr">
@@ -66018,7 +66456,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S816" t="inlineStr"/>
+      <c r="S816" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="817">
       <c r="A817" t="inlineStr">
@@ -66061,7 +66501,7 @@
       </c>
       <c r="K817" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L817" t="inlineStr">
@@ -66257,7 +66697,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S819" t="inlineStr"/>
+      <c r="S819" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="820">
       <c r="A820" t="inlineStr">
@@ -66417,7 +66859,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S821" t="inlineStr"/>
+      <c r="S821" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="822">
       <c r="A822" t="inlineStr">
@@ -67225,7 +67669,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S831" t="inlineStr"/>
+      <c r="S831" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="832">
       <c r="A832" t="inlineStr">
@@ -67304,7 +67750,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S832" t="inlineStr"/>
+      <c r="S832" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="833">
       <c r="A833" t="inlineStr">
@@ -67464,7 +67912,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S834" t="inlineStr"/>
+      <c r="S834" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="835">
       <c r="A835" t="inlineStr">
@@ -67588,7 +68038,7 @@
       </c>
       <c r="K836" t="inlineStr">
         <is>
-          <t>Belirtilmemiş</t>
+          <t>DDR5</t>
         </is>
       </c>
       <c r="L836" t="inlineStr">
@@ -67703,7 +68153,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S837" t="inlineStr"/>
+      <c r="S837" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="838">
       <c r="A838" t="inlineStr">
@@ -67944,7 +68396,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S840" t="inlineStr"/>
+      <c r="S840" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="841">
       <c r="A841" t="inlineStr">
@@ -68426,7 +68880,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S846" t="inlineStr"/>
+      <c r="S846" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="847">
       <c r="A847" t="inlineStr">
@@ -68505,7 +68961,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S847" t="inlineStr"/>
+      <c r="S847" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="848">
       <c r="A848" t="inlineStr">
@@ -68584,7 +69042,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S848" t="inlineStr"/>
+      <c r="S848" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="849">
       <c r="A849" t="inlineStr">
@@ -68663,7 +69123,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S849" t="inlineStr"/>
+      <c r="S849" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="850">
       <c r="A850" t="inlineStr">
@@ -68742,7 +69204,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S850" t="inlineStr"/>
+      <c r="S850" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="851">
       <c r="A851" t="inlineStr">
@@ -68821,7 +69285,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S851" t="inlineStr"/>
+      <c r="S851" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="852">
       <c r="A852" t="inlineStr">
@@ -69062,7 +69528,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S854" t="inlineStr"/>
+      <c r="S854" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="855">
       <c r="A855" t="inlineStr">
@@ -69141,7 +69609,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S855" t="inlineStr"/>
+      <c r="S855" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="856">
       <c r="A856" t="inlineStr">
@@ -69220,7 +69690,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S856" t="inlineStr"/>
+      <c r="S856" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="857">
       <c r="A857" t="inlineStr">
@@ -69542,7 +70014,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S860" t="inlineStr"/>
+      <c r="S860" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="861">
       <c r="A861" t="inlineStr">
@@ -70589,7 +71063,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S873" t="inlineStr"/>
+      <c r="S873" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="874">
       <c r="A874" t="inlineStr">
@@ -70668,7 +71144,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S874" t="inlineStr"/>
+      <c r="S874" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="875">
       <c r="A875" t="inlineStr">
@@ -70990,7 +71468,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S878" t="inlineStr"/>
+      <c r="S878" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="879">
       <c r="A879" t="inlineStr">
@@ -71634,7 +72114,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S886" t="inlineStr"/>
+      <c r="S886" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="887">
       <c r="A887" t="inlineStr">
@@ -71713,7 +72195,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S887" t="inlineStr"/>
+      <c r="S887" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="888">
       <c r="A888" t="inlineStr">
@@ -71792,7 +72276,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S888" t="inlineStr"/>
+      <c r="S888" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="889">
       <c r="A889" t="inlineStr">
@@ -71871,7 +72357,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S889" t="inlineStr"/>
+      <c r="S889" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="890">
       <c r="A890" t="inlineStr">
@@ -72112,7 +72600,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S892" t="inlineStr"/>
+      <c r="S892" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
@@ -72191,7 +72681,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S893" t="inlineStr"/>
+      <c r="S893" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="894">
       <c r="A894" t="inlineStr">
@@ -72270,7 +72762,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S894" t="inlineStr"/>
+      <c r="S894" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="895">
       <c r="A895" t="inlineStr">
@@ -72349,7 +72843,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S895" t="inlineStr"/>
+      <c r="S895" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="896">
       <c r="A896" t="inlineStr">
@@ -72428,7 +72924,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S896" t="inlineStr"/>
+      <c r="S896" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="897">
       <c r="A897" t="inlineStr">
@@ -72507,7 +73005,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S897" t="inlineStr"/>
+      <c r="S897" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="898">
       <c r="A898" t="inlineStr">
@@ -72586,7 +73086,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S898" t="inlineStr"/>
+      <c r="S898" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="899">
       <c r="A899" t="inlineStr">
@@ -72665,7 +73167,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S899" t="inlineStr"/>
+      <c r="S899" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="900">
       <c r="A900" t="inlineStr">
@@ -72744,7 +73248,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S900" t="inlineStr"/>
+      <c r="S900" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="901">
       <c r="A901" t="inlineStr">
@@ -72823,7 +73329,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S901" t="inlineStr"/>
+      <c r="S901" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="902">
       <c r="A902" t="inlineStr">
@@ -72902,7 +73410,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S902" t="inlineStr"/>
+      <c r="S902" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="903">
       <c r="A903" t="inlineStr">
@@ -72981,7 +73491,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S903" t="inlineStr"/>
+      <c r="S903" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="904">
       <c r="A904" t="inlineStr">
@@ -73060,7 +73572,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S904" t="inlineStr"/>
+      <c r="S904" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="905">
       <c r="A905" t="inlineStr">
@@ -73139,7 +73653,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S905" t="inlineStr"/>
+      <c r="S905" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="906">
       <c r="A906" t="inlineStr">
@@ -73218,7 +73734,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S906" t="inlineStr"/>
+      <c r="S906" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="907">
       <c r="A907" t="inlineStr">
@@ -73378,7 +73896,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S908" t="inlineStr"/>
+      <c r="S908" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="909">
       <c r="A909" t="inlineStr">
@@ -73457,7 +73977,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S909" t="inlineStr"/>
+      <c r="S909" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="910">
       <c r="A910" t="inlineStr">
@@ -73617,7 +74139,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S911" t="inlineStr"/>
+      <c r="S911" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="912">
       <c r="A912" t="inlineStr">
@@ -73696,7 +74220,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S912" t="inlineStr"/>
+      <c r="S912" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="913">
       <c r="A913" t="inlineStr">
@@ -73775,7 +74301,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S913" t="inlineStr"/>
+      <c r="S913" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="914">
       <c r="A914" t="inlineStr">
@@ -73854,7 +74382,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S914" t="inlineStr"/>
+      <c r="S914" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="915">
       <c r="A915" t="inlineStr">
@@ -73933,7 +74463,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S915" t="inlineStr"/>
+      <c r="S915" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="916">
       <c r="A916" t="inlineStr">
@@ -74012,7 +74544,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S916" t="inlineStr"/>
+      <c r="S916" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="917">
       <c r="A917" t="inlineStr">
@@ -74091,7 +74625,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S917" t="inlineStr"/>
+      <c r="S917" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="918">
       <c r="A918" t="inlineStr">
@@ -74251,7 +74787,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S919" t="inlineStr"/>
+      <c r="S919" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="920">
       <c r="A920" t="inlineStr">
@@ -74492,7 +75030,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S922" t="inlineStr"/>
+      <c r="S922" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="923">
       <c r="A923" t="inlineStr">
@@ -74571,7 +75111,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S923" t="inlineStr"/>
+      <c r="S923" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="924">
       <c r="A924" t="inlineStr">
@@ -74812,7 +75354,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S926" t="inlineStr"/>
+      <c r="S926" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="927">
       <c r="A927" t="inlineStr">
@@ -74891,7 +75435,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S927" t="inlineStr"/>
+      <c r="S927" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="928">
       <c r="A928" t="inlineStr">
@@ -74970,7 +75516,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S928" t="inlineStr"/>
+      <c r="S928" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="929">
       <c r="A929" t="inlineStr">
@@ -75211,7 +75759,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S931" t="inlineStr"/>
+      <c r="S931" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="932">
       <c r="A932" t="inlineStr">
@@ -75290,7 +75840,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S932" t="inlineStr"/>
+      <c r="S932" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="933">
       <c r="A933" t="inlineStr">
@@ -75369,7 +75921,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S933" t="inlineStr"/>
+      <c r="S933" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="934">
       <c r="A934" t="inlineStr">
@@ -75529,7 +76083,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S935" t="inlineStr"/>
+      <c r="S935" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="936">
       <c r="A936" t="inlineStr">
@@ -75608,7 +76164,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S936" t="inlineStr"/>
+      <c r="S936" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="937">
       <c r="A937" t="inlineStr">
@@ -75687,7 +76245,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S937" t="inlineStr"/>
+      <c r="S937" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="938">
       <c r="A938" t="inlineStr">
@@ -75766,7 +76326,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S938" t="inlineStr"/>
+      <c r="S938" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="939">
       <c r="A939" t="inlineStr">
@@ -75845,7 +76407,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S939" t="inlineStr"/>
+      <c r="S939" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="940">
       <c r="A940" t="inlineStr">
@@ -75924,7 +76488,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S940" t="inlineStr"/>
+      <c r="S940" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="941">
       <c r="A941" t="inlineStr">
@@ -76003,7 +76569,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S941" t="inlineStr"/>
+      <c r="S941" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="942">
       <c r="A942" t="inlineStr">
@@ -76082,7 +76650,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S942" t="inlineStr"/>
+      <c r="S942" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="943">
       <c r="A943" t="inlineStr">
@@ -76161,7 +76731,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S943" t="inlineStr"/>
+      <c r="S943" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="944">
       <c r="A944" t="inlineStr">
@@ -76240,7 +76812,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S944" t="inlineStr"/>
+      <c r="S944" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="945">
       <c r="A945" t="inlineStr">
@@ -76319,7 +76893,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S945" t="inlineStr"/>
+      <c r="S945" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="946">
       <c r="A946" t="inlineStr">
@@ -76398,7 +76974,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S946" t="inlineStr"/>
+      <c r="S946" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="947">
       <c r="A947" t="inlineStr">
@@ -76477,7 +77055,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S947" t="inlineStr"/>
+      <c r="S947" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="948">
       <c r="A948" t="inlineStr">
@@ -76556,7 +77136,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S948" t="inlineStr"/>
+      <c r="S948" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="949">
       <c r="A949" t="inlineStr">
@@ -76635,7 +77217,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S949" t="inlineStr"/>
+      <c r="S949" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="950">
       <c r="A950" t="inlineStr">
@@ -76714,7 +77298,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S950" t="inlineStr"/>
+      <c r="S950" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="951">
       <c r="A951" t="inlineStr">
@@ -76793,7 +77379,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S951" t="inlineStr"/>
+      <c r="S951" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="952">
       <c r="A952" t="inlineStr">
@@ -76872,7 +77460,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S952" t="inlineStr"/>
+      <c r="S952" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="953">
       <c r="A953" t="inlineStr">
@@ -76951,7 +77541,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S953" t="inlineStr"/>
+      <c r="S953" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="954">
       <c r="A954" t="inlineStr">
@@ -77030,7 +77622,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S954" t="inlineStr"/>
+      <c r="S954" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="955">
       <c r="A955" t="inlineStr">
@@ -77109,7 +77703,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S955" t="inlineStr"/>
+      <c r="S955" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="956">
       <c r="A956" t="inlineStr">
@@ -77188,7 +77784,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S956" t="inlineStr"/>
+      <c r="S956" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="957">
       <c r="A957" t="inlineStr">
@@ -77267,7 +77865,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S957" t="inlineStr"/>
+      <c r="S957" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="958">
       <c r="A958" t="inlineStr">
@@ -77346,7 +77946,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S958" t="inlineStr"/>
+      <c r="S958" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="959">
       <c r="A959" t="inlineStr">
@@ -77425,7 +78027,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S959" t="inlineStr"/>
+      <c r="S959" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="960">
       <c r="A960" t="inlineStr">
@@ -77504,7 +78108,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S960" t="inlineStr"/>
+      <c r="S960" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="961">
       <c r="A961" t="inlineStr">
@@ -77583,7 +78189,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S961" t="inlineStr"/>
+      <c r="S961" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="962">
       <c r="A962" t="inlineStr">
@@ -77662,7 +78270,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S962" t="inlineStr"/>
+      <c r="S962" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="963">
       <c r="A963" t="inlineStr">
@@ -77741,7 +78351,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S963" t="inlineStr"/>
+      <c r="S963" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="964">
       <c r="A964" t="inlineStr">
@@ -77820,7 +78432,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S964" t="inlineStr"/>
+      <c r="S964" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="965">
       <c r="A965" t="inlineStr">
@@ -77899,7 +78513,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S965" t="inlineStr"/>
+      <c r="S965" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="966">
       <c r="A966" t="inlineStr">
@@ -77978,7 +78594,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S966" t="inlineStr"/>
+      <c r="S966" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="967">
       <c r="A967" t="inlineStr">
@@ -78057,7 +78675,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S967" t="inlineStr"/>
+      <c r="S967" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="968">
       <c r="A968" t="inlineStr">
@@ -78136,7 +78756,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S968" t="inlineStr"/>
+      <c r="S968" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="969">
       <c r="A969" t="inlineStr">
@@ -78215,7 +78837,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S969" t="inlineStr"/>
+      <c r="S969" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="970">
       <c r="A970" t="inlineStr">
@@ -78294,7 +78918,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S970" t="inlineStr"/>
+      <c r="S970" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="971">
       <c r="A971" t="inlineStr">
@@ -78373,7 +78999,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S971" t="inlineStr"/>
+      <c r="S971" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="972">
       <c r="A972" t="inlineStr">
@@ -78452,7 +79080,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S972" t="inlineStr"/>
+      <c r="S972" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="973">
       <c r="A973" t="inlineStr">
@@ -78531,7 +79161,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S973" t="inlineStr"/>
+      <c r="S973" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="974">
       <c r="A974" t="inlineStr">
@@ -78610,7 +79242,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S974" t="inlineStr"/>
+      <c r="S974" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="975">
       <c r="A975" t="inlineStr">
@@ -78689,7 +79323,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S975" t="inlineStr"/>
+      <c r="S975" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="976">
       <c r="A976" t="inlineStr">
@@ -78768,7 +79404,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S976" t="inlineStr"/>
+      <c r="S976" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="977">
       <c r="A977" t="inlineStr">
@@ -78847,7 +79485,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S977" t="inlineStr"/>
+      <c r="S977" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="978">
       <c r="A978" t="inlineStr">
@@ -78926,7 +79566,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S978" t="inlineStr"/>
+      <c r="S978" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="979">
       <c r="A979" t="inlineStr">
@@ -79005,7 +79647,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S979" t="inlineStr"/>
+      <c r="S979" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="980">
       <c r="A980" t="inlineStr">
@@ -79084,7 +79728,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S980" t="inlineStr"/>
+      <c r="S980" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="981">
       <c r="A981" t="inlineStr">
@@ -79163,7 +79809,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S981" t="inlineStr"/>
+      <c r="S981" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="982">
       <c r="A982" t="inlineStr">
@@ -79242,7 +79890,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S982" t="inlineStr"/>
+      <c r="S982" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="983">
       <c r="A983" t="inlineStr">
@@ -79321,7 +79971,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S983" t="inlineStr"/>
+      <c r="S983" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="984">
       <c r="A984" t="inlineStr">
@@ -79481,7 +80133,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S985" t="inlineStr"/>
+      <c r="S985" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="986">
       <c r="A986" t="inlineStr">
@@ -79560,7 +80214,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S986" t="inlineStr"/>
+      <c r="S986" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="987">
       <c r="A987" t="inlineStr">
@@ -79639,7 +80295,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S987" t="inlineStr"/>
+      <c r="S987" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="988">
       <c r="A988" t="inlineStr">
@@ -79718,7 +80376,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S988" t="inlineStr"/>
+      <c r="S988" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="989">
       <c r="A989" t="inlineStr">
@@ -79797,7 +80457,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S989" t="inlineStr"/>
+      <c r="S989" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="990">
       <c r="A990" t="inlineStr">
@@ -79876,7 +80538,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S990" t="inlineStr"/>
+      <c r="S990" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="991">
       <c r="A991" t="inlineStr">
@@ -79955,7 +80619,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S991" t="inlineStr"/>
+      <c r="S991" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="992">
       <c r="A992" t="inlineStr">
@@ -80844,7 +81510,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1002" t="inlineStr"/>
+      <c r="S1002" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1003">
       <c r="A1003" t="inlineStr">
@@ -80923,7 +81591,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1003" t="inlineStr"/>
+      <c r="S1003" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1004">
       <c r="A1004" t="inlineStr">
@@ -81002,7 +81672,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1004" t="inlineStr"/>
+      <c r="S1004" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1005">
       <c r="A1005" t="inlineStr">
@@ -81081,7 +81753,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1005" t="inlineStr"/>
+      <c r="S1005" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1006">
       <c r="A1006" t="inlineStr">
@@ -81160,7 +81834,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1006" t="inlineStr"/>
+      <c r="S1006" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1007">
       <c r="A1007" t="inlineStr">
@@ -81239,7 +81915,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1007" t="inlineStr"/>
+      <c r="S1007" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1008">
       <c r="A1008" t="inlineStr">
@@ -81318,7 +81996,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1008" t="inlineStr"/>
+      <c r="S1008" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1009">
       <c r="A1009" t="inlineStr">
@@ -81397,7 +82077,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1009" t="inlineStr"/>
+      <c r="S1009" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1010">
       <c r="A1010" t="inlineStr">
@@ -81476,7 +82158,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1010" t="inlineStr"/>
+      <c r="S1010" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1011">
       <c r="A1011" t="inlineStr">
@@ -81555,7 +82239,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1011" t="inlineStr"/>
+      <c r="S1011" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1012">
       <c r="A1012" t="inlineStr">
@@ -81634,7 +82320,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1012" t="inlineStr"/>
+      <c r="S1012" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1013">
       <c r="A1013" t="inlineStr">
@@ -81713,7 +82401,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1013" t="inlineStr"/>
+      <c r="S1013" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1014">
       <c r="A1014" t="inlineStr">
@@ -81792,7 +82482,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1014" t="inlineStr"/>
+      <c r="S1014" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1015">
       <c r="A1015" t="inlineStr">
@@ -81871,7 +82563,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1015" t="inlineStr"/>
+      <c r="S1015" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1016">
       <c r="A1016" t="inlineStr">
@@ -81950,7 +82644,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1016" t="inlineStr"/>
+      <c r="S1016" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1017">
       <c r="A1017" t="inlineStr">
@@ -82191,7 +82887,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1019" t="inlineStr"/>
+      <c r="S1019" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1020">
       <c r="A1020" t="inlineStr">
@@ -82270,7 +82968,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1020" t="inlineStr"/>
+      <c r="S1020" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1021">
       <c r="A1021" t="inlineStr">
@@ -82349,7 +83049,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1021" t="inlineStr"/>
+      <c r="S1021" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1022">
       <c r="A1022" t="inlineStr">
@@ -82744,7 +83446,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1026" t="inlineStr"/>
+      <c r="S1026" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1027">
       <c r="A1027" t="inlineStr">
@@ -82823,7 +83527,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1027" t="inlineStr"/>
+      <c r="S1027" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1028">
       <c r="A1028" t="inlineStr">
@@ -82902,7 +83608,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1028" t="inlineStr"/>
+      <c r="S1028" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1029">
       <c r="A1029" t="inlineStr">
@@ -87193,7 +87901,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1081" t="inlineStr"/>
+      <c r="S1081" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1082">
       <c r="A1082" t="inlineStr">
@@ -87272,7 +87982,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1082" t="inlineStr"/>
+      <c r="S1082" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1083">
       <c r="A1083" t="inlineStr">
@@ -87918,7 +88630,9 @@
           <t>Linux</t>
         </is>
       </c>
-      <c r="S1090" t="inlineStr"/>
+      <c r="S1090" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1091">
       <c r="A1091" t="inlineStr">
@@ -87997,7 +88711,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1091" t="inlineStr"/>
+      <c r="S1091" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1092">
       <c r="A1092" t="inlineStr">
@@ -88236,7 +88952,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1094" t="inlineStr"/>
+      <c r="S1094" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1095">
       <c r="A1095" t="inlineStr">
@@ -88315,7 +89033,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1095" t="inlineStr"/>
+      <c r="S1095" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1096">
       <c r="A1096" t="inlineStr">
@@ -88475,7 +89195,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1097" t="inlineStr"/>
+      <c r="S1097" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1098">
       <c r="A1098" t="inlineStr">
@@ -88554,7 +89276,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1098" t="inlineStr"/>
+      <c r="S1098" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1099">
       <c r="A1099" t="inlineStr">
@@ -92602,7 +93326,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1148" t="inlineStr"/>
+      <c r="S1148" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1149">
       <c r="A1149" t="inlineStr">
@@ -92681,7 +93407,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1149" t="inlineStr"/>
+      <c r="S1149" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1150">
       <c r="A1150" t="inlineStr">
@@ -92841,7 +93569,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1151" t="inlineStr"/>
+      <c r="S1151" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1152">
       <c r="A1152" t="inlineStr">
@@ -92920,7 +93650,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1152" t="inlineStr"/>
+      <c r="S1152" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1153">
       <c r="A1153" t="inlineStr">
@@ -92999,7 +93731,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1153" t="inlineStr"/>
+      <c r="S1153" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1154">
       <c r="A1154" t="inlineStr">
@@ -93078,7 +93812,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1154" t="inlineStr"/>
+      <c r="S1154" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1155">
       <c r="A1155" t="inlineStr">
@@ -93157,7 +93893,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1155" t="inlineStr"/>
+      <c r="S1155" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1156">
       <c r="A1156" t="inlineStr">
@@ -93236,7 +93974,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1156" t="inlineStr"/>
+      <c r="S1156" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1157">
       <c r="A1157" t="inlineStr">
@@ -93315,7 +94055,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1157" t="inlineStr"/>
+      <c r="S1157" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1158">
       <c r="A1158" t="inlineStr">
@@ -93394,7 +94136,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1158" t="inlineStr"/>
+      <c r="S1158" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1159">
       <c r="A1159" t="inlineStr">
@@ -93473,7 +94217,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1159" t="inlineStr"/>
+      <c r="S1159" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1160">
       <c r="A1160" t="inlineStr">
@@ -93552,7 +94298,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1160" t="inlineStr"/>
+      <c r="S1160" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1161">
       <c r="A1161" t="inlineStr">
@@ -93631,7 +94379,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1161" t="inlineStr"/>
+      <c r="S1161" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1162">
       <c r="A1162" t="inlineStr">
@@ -93710,7 +94460,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1162" t="inlineStr"/>
+      <c r="S1162" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1163">
       <c r="A1163" t="inlineStr">
@@ -93789,7 +94541,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1163" t="inlineStr"/>
+      <c r="S1163" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1164">
       <c r="A1164" t="inlineStr">
@@ -93868,7 +94622,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1164" t="inlineStr"/>
+      <c r="S1164" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1165">
       <c r="A1165" t="inlineStr">
@@ -93947,7 +94703,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1165" t="inlineStr"/>
+      <c r="S1165" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1166">
       <c r="A1166" t="inlineStr">
@@ -94026,7 +94784,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1166" t="inlineStr"/>
+      <c r="S1166" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1167">
       <c r="A1167" t="inlineStr">
@@ -94105,7 +94865,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1167" t="inlineStr"/>
+      <c r="S1167" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1168">
       <c r="A1168" t="inlineStr">
@@ -94184,7 +94946,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1168" t="inlineStr"/>
+      <c r="S1168" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1169">
       <c r="A1169" t="inlineStr">
@@ -94263,7 +95027,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1169" t="inlineStr"/>
+      <c r="S1169" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1170">
       <c r="A1170" t="inlineStr">
@@ -94342,7 +95108,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1170" t="inlineStr"/>
+      <c r="S1170" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1171">
       <c r="A1171" t="inlineStr">
@@ -94421,7 +95189,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1171" t="inlineStr"/>
+      <c r="S1171" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1172">
       <c r="A1172" t="inlineStr">
@@ -94500,7 +95270,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1172" t="inlineStr"/>
+      <c r="S1172" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1173">
       <c r="A1173" t="inlineStr">
@@ -94579,7 +95351,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1173" t="inlineStr"/>
+      <c r="S1173" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1174">
       <c r="A1174" t="inlineStr">
@@ -94658,7 +95432,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1174" t="inlineStr"/>
+      <c r="S1174" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1175">
       <c r="A1175" t="inlineStr">
@@ -94737,7 +95513,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1175" t="inlineStr"/>
+      <c r="S1175" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1176">
       <c r="A1176" t="inlineStr">
@@ -94816,7 +95594,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1176" t="inlineStr"/>
+      <c r="S1176" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1177">
       <c r="A1177" t="inlineStr">
@@ -94895,7 +95675,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1177" t="inlineStr"/>
+      <c r="S1177" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1178">
       <c r="A1178" t="inlineStr">
@@ -94974,7 +95756,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1178" t="inlineStr"/>
+      <c r="S1178" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1179">
       <c r="A1179" t="inlineStr">
@@ -95053,7 +95837,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1179" t="inlineStr"/>
+      <c r="S1179" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1180">
       <c r="A1180" t="inlineStr">
@@ -95132,7 +95918,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1180" t="inlineStr"/>
+      <c r="S1180" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1181">
       <c r="A1181" t="inlineStr">
@@ -95211,7 +95999,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1181" t="inlineStr"/>
+      <c r="S1181" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1182">
       <c r="A1182" t="inlineStr">
@@ -95290,7 +96080,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1182" t="inlineStr"/>
+      <c r="S1182" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1183">
       <c r="A1183" t="inlineStr">
@@ -95369,7 +96161,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1183" t="inlineStr"/>
+      <c r="S1183" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1184">
       <c r="A1184" t="inlineStr">
@@ -95448,7 +96242,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1184" t="inlineStr"/>
+      <c r="S1184" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1185">
       <c r="A1185" t="inlineStr">
@@ -95527,7 +96323,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1185" t="inlineStr"/>
+      <c r="S1185" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1186">
       <c r="A1186" t="inlineStr">
@@ -95606,7 +96404,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1186" t="inlineStr"/>
+      <c r="S1186" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1187">
       <c r="A1187" t="inlineStr">
@@ -95685,7 +96485,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1187" t="inlineStr"/>
+      <c r="S1187" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1188">
       <c r="A1188" t="inlineStr">
@@ -95764,7 +96566,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1188" t="inlineStr"/>
+      <c r="S1188" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1189">
       <c r="A1189" t="inlineStr">
@@ -95843,7 +96647,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1189" t="inlineStr"/>
+      <c r="S1189" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1190">
       <c r="A1190" t="inlineStr">
@@ -95922,7 +96728,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1190" t="inlineStr"/>
+      <c r="S1190" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1191">
       <c r="A1191" t="inlineStr">
@@ -96001,7 +96809,9 @@
           <t>Free Dos</t>
         </is>
       </c>
-      <c r="S1191" t="inlineStr"/>
+      <c r="S1191" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1192">
       <c r="A1192" t="inlineStr">
@@ -96080,7 +96890,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1192" t="inlineStr"/>
+      <c r="S1192" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1193">
       <c r="A1193" t="inlineStr">
@@ -96159,7 +96971,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1193" t="inlineStr"/>
+      <c r="S1193" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1194">
       <c r="A1194" t="inlineStr">
@@ -96238,7 +97052,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1194" t="inlineStr"/>
+      <c r="S1194" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1195">
       <c r="A1195" t="inlineStr">
@@ -96317,7 +97133,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1195" t="inlineStr"/>
+      <c r="S1195" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1196">
       <c r="A1196" t="inlineStr">
@@ -96396,7 +97214,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1196" t="inlineStr"/>
+      <c r="S1196" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1197">
       <c r="A1197" t="inlineStr">
@@ -96475,7 +97295,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1197" t="inlineStr"/>
+      <c r="S1197" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1198">
       <c r="A1198" t="inlineStr">
@@ -96635,7 +97457,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1199" t="inlineStr"/>
+      <c r="S1199" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1200">
       <c r="A1200" t="inlineStr">
@@ -96714,7 +97538,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1200" t="inlineStr"/>
+      <c r="S1200" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
     <row r="1201">
       <c r="A1201" t="inlineStr">
@@ -96793,7 +97619,9 @@
           <t>Windows</t>
         </is>
       </c>
-      <c r="S1201" t="inlineStr"/>
+      <c r="S1201" t="n">
+        <v>48.7393727735369</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>